<commit_message>
feat(F-NAR-019): ATOM-DIF.BES.002-05 Le garage en carton
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.BES.002-05.xlsx
+++ b/stories/arbres/ATOM-DIF.BES.002-05.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Chouchou veut que la voiture rouge rentre dans un garage en carton. Il propose. Mila dit non, puis je regarde, puis plus tard. Le rabat est dur, il le plie deux fois. Chouchou accepte. La voiture fait toc. Le rabat se ferme.</t>
+          <t>La cheminée boit le vent. Sur la brique, un éclat de cheminée brille. Un carton ouvert attend dans le couloir. Chouchou veut la voiture rouge dans le garage maintenant. Elle tire trop vite, attrape Mila : non. Le rabat est dur, l'éclat glisse. Elle refuse de foncer, propose. Mila regarde, plus tard. Merci vécu. La voiture file trop vite. Elle refuse, propose le rabat. Toc. L'éclat de cheminée tient.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le vent chante dans la cheminée. Ça fait un son long, tout bas. Un carton ouvert attend dans le couloir. Il sent encore le crayon. Un trait bleu reste sur un bord. Une voiture rouge de bois est par terre. Ses roues sont noires et lisses. Un phare est peint en jaune. Tu entends le vent, Chouchou ? Oui, maman. J'ai plié un rabat, tout à l'heure. Ça peut être une porte. On reste au couloir, d'accord ? D'accord. La voiture rentre dedans. En ce moment, Chouchou tire le carton. Le carton racle un peu le sol. Une poussière s'envole, toute légère. Maman ouvre la porte. Mila arrive. Elle a des chaussettes à rayures. Tu viens ? Non. Chouchou regarde papa. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. D'accord. Chouchou pousse le rabat. Le rabat est dur. Le rabat est dur, hein ? Oui. Il le plie une fois. Le carton craque, tout doux. Puis une autre fois. Le rabat s'ouvre mieux. Plus tard, tu viens ? Je regarde. Regarder, c'est une réponse.</t>
+          <t>La cheminée boit le vent, froid et creux. Ça souffle, papa ! Tu l'entends, dans la brique ? Oui, un son long. Sur la brique, un éclat de cheminée brille. Il brille, maman. C'est le vent, sur la brique ? Oui, un petit point. Le carrelage du couloir est froid sous les chaussettes. Il pique les pieds. On reste près du carton ? Oui, papa. Un carton ouvert attend contre le mur. Il sent le papier neuf. Ça sent le papier. Le rabat peut faire une porte. Une porte de garage ! Une voiture rouge de bois est par terre. Ses roues sont noires et lisses. Le phare est jaune. Tu la vois, Chouchou ? Oui, elle rentre dedans, maintenant ! Maman ouvre la porte du couloir. Mila arrive, en chaussettes à rayures. Mila ! J'arrive. Tes chaussettes ont des rayures ? Oui. Le garage, maintenant, Mila ! En ce moment, Chouchou tire le carton trop vite. Le carton racle le carrelage. Une poussière s'envole. Tu viens, tout de suite ! Chouchou attrape la manche de Mila. Non. Mila recule vers le mur. Oh. Chouchou pousse le rabat d'un coup. Le rabat est dur, il résiste. Le rabat est dur, Chouchou ? Oui. La voiture tape le bord. Elle ne rentre pas. Oh. L'éclat de cheminée glisse sur la brique. Il part. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à Mila, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le vent. Personne n'entend la fin. Chouchou referme la bouche, un instant. La voiture reste dehors, un peu lourde.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le vent chante dans la cheminée. Ça fait un son long, tout bas. Un carton ouvert attend dans le couloir. Il sent encore le crayon. Un trait bleu reste sur un bord. Une voiture rouge de bois est par terre. Ses roues sont noires et lisses. Un phare est peint en jaune. Tu entends le vent, Chouchou ? Oui, maman. J'ai plié un rabat, tout à l'heure. Ça peut être une porte. On reste au couloir, d'accord ? D'accord. La voiture rentre dedans. En ce moment, Chouchou tire le carton. Le carton racle un peu le sol. Une poussière s'envole, toute légère. Maman ouvre la porte. Mila arrive. Elle a des chaussettes à rayures. Tu viens ? Non. Chouchou regarde papa. On peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. D'accord. Chouchou pousse le rabat. Le rabat est dur. Le rabat est dur, hein ? Oui. Il le plie une fois. Le carton craque, tout doux. Puis une autre fois. Le rabat s'ouvre mieux. Plus tard, tu viens ? Je regarde. Regarder, c'est une réponse.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La cheminée boit le vent, froid et creux. Ça souffle, papa ! Tu l'entends, dans la brique ? Oui, un son long. Sur la brique, un &lt;emphasis level="moderate"&gt;éclat de cheminée&lt;/emphasis&gt; brille. Il brille, maman. C'est le vent, sur la brique ? Oui, un petit point. Le carrelage du couloir est froid sous les chaussettes. Il pique les pieds. On reste près du carton ? Oui, papa. Un carton ouvert attend contre le mur. Il sent le papier neuf. Ça sent le papier. Le rabat peut faire une porte. Une porte de garage ! Une voiture rouge de bois est par terre. Ses roues sont noires et lisses. Le phare est jaune. Tu la vois, Chouchou ? Oui, elle rentre dedans, maintenant ! Maman ouvre la porte du couloir. Mila arrive, en chaussettes à rayures. Mila ! J'arrive. Tes chaussettes ont des rayures ? Oui. Le garage, maintenant, Mila ! En ce moment, Chouchou tire le carton trop vite. Le carton racle le carrelage. Une poussière s'envole. Tu viens, tout de suite ! Chouchou attrape la manche de Mila. Non. Mila recule vers le mur. Oh. Chouchou pousse le rabat d'un coup. Le rabat est dur, il résiste. Le rabat est dur, Chouchou ? Oui. La voiture tape le bord. Elle ne rentre pas. Oh. L'éclat de cheminée glisse sur la brique. Il part. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à Mila, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le vent. Personne n'entend la fin. Chouchou referme la bouche, un instant. La voiture reste dehors, un peu lourde.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Kilian est dans le salon. Les coussins sont par terre. Maman ouvre la porte. Maël arrive. Kilian veut faire une cabane. Il va &lt;emphasis&gt;proposer&lt;/emphasis&gt; un jeu. Kilian dit : tu viens ? Maël dit : non. Kilian regarde maman. Maman dit : on peut proposer. On peut accepter plusieurs réponses. Oui. Non. Regarder. Plus tard. Kilian dit : d'accord. Il pose un coussin. Maël s'assoit près du canapé. Il regarde. Kilian laisse Maël à sa place. Il propose encore, tout doux. Kilian dit : plus tard, tu viens ? Maël dit : je regarde. Maman sourit. Maman dit : regarder, c'est une réponse. On peut accepter plusieurs réponses. Kilian pose un autre coussin. La cabane grandit. Maël avance un peu. Il ne touche pas. C'est bien. Kilian dit : tu veux un coussin ? Maël dit : plus tard. Kilian dit : d'accord. Il continue. Maman chante tout bas. Maman dit : tu as su proposer. Tu as su accepter. Plusieurs réponses sont possibles. [pause]</t>
+          <t>La cheminée boit le vent, froid et creux. Ça souffle, papa ! Tu l'entends, dans la brique ? Oui, un son long. Sur la brique, un &lt;emphasis&gt;éclat de cheminée&lt;/emphasis&gt; brille. Il brille, maman. C'est le vent, sur la brique ? Oui, un petit point. Le carrelage du couloir est froid sous les chaussettes. Il pique les pieds. On reste près du carton ? Oui, papa. Un carton ouvert attend contre le mur. Il sent le papier neuf. Ça sent le papier. Le rabat peut faire une porte. Une porte de garage ! Une voiture rouge de bois est par terre. Ses roues sont noires et lisses. Le phare est jaune. Tu la vois, Chouchou ? Oui, elle rentre dedans, maintenant ! Maman ouvre la porte du couloir. Mila arrive, en chaussettes à rayures. Mila ! J'arrive. Tes chaussettes ont des rayures ? Oui. Le garage, maintenant, Mila ! En ce moment, Chouchou tire le carton trop vite. Le carton racle le carrelage. Une poussière s'envole. Tu viens, tout de suite ! Chouchou attrape la manche de Mila. Non. Mila recule vers le mur. Oh. Chouchou pousse le rabat d'un coup. Le rabat est dur, il résiste. Le rabat est dur, Chouchou ? Oui. La voiture tape le bord. Elle ne rentre pas. Oh. L'éclat de cheminée glisse sur la brique. Il part. Le sourire de Chouchou disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Tu parles à Mila, Chouchou ? Papa s'accroupit à la même hauteur. Oui, papa. La phrase se perd dans le vent. Personne n'entend la fin. Chouchou referme la bouche, un instant. La voiture reste dehors, un peu lourde. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>éclat de cheminée</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,51 +1326,68 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_garage_avec_mila_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le vent chante dans la cheminée.
-narrateur|Ça fait un son long, tout bas.
-narrateur|Un carton ouvert attend dans le couloir.
-narrateur|Il sent encore le crayon.
-narrateur|Un trait bleu reste sur un bord.
+          <t>narrateur|La cheminée boit le vent, froid et creux.
+enfant-f|Ça souffle, papa !
+papa|Tu l'entends, dans la brique ?
+enfant-f|Oui, un son long.
+narrateur|Sur la brique, un éclat de cheminée brille.
+enfant-f|Il brille, maman.
+maman|C'est le vent, sur la brique ?
+enfant-f|Oui, un petit point.
+narrateur|Le carrelage du couloir est froid sous les chaussettes.
+enfant-f|Il pique les pieds.
+papa|On reste près du carton ?
+enfant-f|Oui, papa.
+narrateur|Un carton ouvert attend contre le mur.
+narrateur|Il sent le papier neuf.
+enfant-f|Ça sent le papier.
+maman|Le rabat peut faire une porte.
+enfant-f|Une porte de garage !
 narrateur|Une voiture rouge de bois est par terre.
 narrateur|Ses roues sont noires et lisses.
-narrateur|Un phare est peint en jaune.
-maman|Tu entends le vent, Chouchou ?
-enfant-m|Oui, maman.
-papa|J'ai plié un rabat, tout à l'heure.
-papa|Ça peut être une porte.
-maman|On reste au couloir, d'accord ?
-enfant-m|D'accord.
-enfant-m|La voiture rentre dedans.
-narrateur|En ce moment, Chouchou tire le carton.
-narrateur|Le carton racle un peu le sol.
-narrateur|Une poussière s'envole, toute légère.
-narrateur|Maman ouvre la porte.
-narrateur|Mila arrive.
-narrateur|Elle a des chaussettes à rayures.
-enfant-m|Tu viens ?
+enfant-f|Le phare est jaune.
+papa|Tu la vois, Chouchou ?
+enfant-f|Oui, elle rentre dedans, maintenant !
+narrateur|Maman ouvre la porte du couloir.
+narrateur|Mila arrive, en chaussettes à rayures.
+enfant-f|Mila !
+copine|J'arrive.
+maman|Tes chaussettes ont des rayures ?
+copine|Oui.
+enfant-f|Le garage, maintenant, Mila !
+narrateur|En ce moment, Chouchou tire le carton trop vite.
+narrateur|Le carton racle le carrelage.
+narrateur|Une poussière s'envole.
+enfant-f|Tu viens, tout de suite !
+narrateur|Chouchou attrape la manche de Mila.
 copine|Non.
-narrateur|Chouchou regarde papa.
-papa|On peut proposer.
-maman|On peut accepter plusieurs réponses.
-papa|Oui.
-papa|Non.
-papa|Regarder.
-papa|Plus tard.
-enfant-m|D'accord.
-narrateur|Chouchou pousse le rabat.
-narrateur|Le rabat est dur.
-papa|Le rabat est dur, hein ?
-enfant-m|Oui.
-narrateur|Il le plie une fois.
-narrateur|Le carton craque, tout doux.
-narrateur|Puis une autre fois.
-narrateur|Le rabat s'ouvre mieux.
-enfant-m|Plus tard, tu viens ?
-copine|Je regarde.
-maman|Regarder, c'est une réponse.</t>
+narrateur|Mila recule vers le mur.
+enfant-f|Oh.
+narrateur|Chouchou pousse le rabat d'un coup.
+narrateur|Le rabat est dur, il résiste.
+papa|Le rabat est dur, Chouchou ?
+enfant-f|Oui.
+narrateur|La voiture tape le bord.
+narrateur|Elle ne rentre pas.
+enfant-f|Oh.
+narrateur|L'éclat de cheminée glisse sur la brique.
+enfant-f|Il part.
+narrateur|Le sourire de Chouchou disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+papa|Tu parles à Mila, Chouchou ?
+narrateur|Papa s'accroupit à la même hauteur.
+enfant-f|Oui, papa.
+narrateur|La phrase se perd dans le vent.
+narrateur|Personne n'entend la fin.
+narrateur|Chouchou referme la bouche, un instant.
+narrateur|La voiture reste dehors, un peu lourde.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1407,12 +1424,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Chouchou invite Mila. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Chouchou invite &lt;emphasis level="moderate"&gt;Mila&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Kilian invite Maël. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Chouchou invite &lt;emphasis&gt;Mila&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1437,7 +1454,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>On peut proposer. On peut accepter. Que fait-on ?</t>
+          <t>Chouchou peut proposer. Que fait-on ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1475,7 +1492,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1486,7 +1503,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1501,34 +1518,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Mila</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1543,17 +1564,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_invite_sans_tirer_la_manche; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1586,17 +1607,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a su proposer. Il accepte plusieurs réponses. D'accord. Mila s'assoit près du mur. Elle regarde la voiture. Chouchou pousse la voiture. Les roues font un petit bruit. Le phare jaune avance. Tu as entendu les roues ? Oui, papa. Tu veux pousser ? Plus tard. D'accord. Plusieurs réponses sont possibles. La voiture s'arrête devant le rabat. Le phare jaune touche le carton. Elle n'est pas encore dedans. Tu as plié le rabat. Deux fois. Mila avance un peu. Elle reste à regarder. C'est bien.</t>
+          <t>Chouchou avance la voiture trop vite. Tu pousses, Mila, maintenant ! Les mots se bousculent dans sa bouche. Non. Mila reste près du mur. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle lâche la manche, un peu. La voiture est dehors, Chouchou ? Papa reste à sa hauteur. Le rabat est dur, sous tes mains. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. Tu veux pousser ? Mila ne dit rien. Elle s'assoit près du mur. Je regarde. D'accord. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens la voiture des deux mains ? Oui, maman. Les roues sont froides. Tu parles du vent, si tu veux ? La cheminée boit le vent. On reste au couloir, Chouchou ? Oui. Chouchou pousse la voiture sans presser. Les roues font un petit bruit. Le phare jaune avance. Elle va au rabat. Tu as entendu les roues ? Oui, papa. La voiture s'arrête devant le rabat. Le phare jaune touche le carton. Elle n'est pas dedans. Presque.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Chouchou a su proposer. Il accepte plusieurs réponses. D'accord. Mila s'assoit près du mur. Elle regarde la voiture. Chouchou pousse la voiture. Les roues font un petit bruit. Le phare jaune avance. Tu as entendu les roues ? Oui, papa. Tu veux pousser ? Plus tard. D'accord. Plusieurs réponses sont possibles. La voiture s'arrête devant le rabat. Le phare jaune touche le carton. Elle n'est pas encore dedans. Tu as plié le rabat. Deux fois. Mila avance un peu. Elle reste à regarder. C'est bien.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou avance la voiture trop vite. Tu pousses, Mila, maintenant ! Les mots se bousculent dans sa bouche. Non. Mila reste près du mur. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle lâche la manche, un peu. La voiture est dehors, Chouchou ? Papa reste à sa hauteur. Le rabat est dur, sous tes mains. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. &lt;emphasis level="moderate"&gt;Tu veux pousser&lt;/emphasis&gt; ? Mila ne dit rien. Elle s'assoit près du mur. Je regarde. D'accord. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens la voiture des deux mains ? Oui, maman. Les roues sont froides. Tu parles du vent, si tu veux ? La cheminée boit le vent. On reste au couloir, Chouchou ? Oui. Chouchou pousse la voiture sans presser. Les roues font un petit bruit. Le phare jaune avance. Elle va au rabat. Tu as entendu les roues ? Oui, papa. La voiture s'arrête devant le rabat. Le phare jaune touche le carton. Elle n'est pas dedans. Presque.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Kilian a su &lt;emphasis&gt;proposer&lt;/emphasis&gt;. Maël a dit non, puis regarder. Kilian a pu accepter plusieurs réponses. [pause]</t>
+          <t>Chouchou avance la voiture trop vite. Tu pousses, Mila, maintenant ! Les mots se bousculent dans sa bouche. Non. Mila reste près du mur. Oh. Le sourire ne revient pas. Chouchou refuse de foncer. Elle lâche la manche, un peu. La voiture est dehors, Chouchou ? Papa reste à sa hauteur. Le rabat est dur, sous tes mains. Maman n'a pas fini non plus. Chouchou attend que le silence arrive. &lt;emphasis&gt;Tu veux pousser&lt;/emphasis&gt; ? Mila ne dit rien. Elle s'assoit près du mur. Je regarde. D'accord. Merci, Chouchou. Papa a entendu toute la phrase. Tu tiens la voiture des deux mains ? Oui, maman. Les roues sont froides. Tu parles du vent, si tu veux ? La cheminée boit le vent. On reste au couloir, Chouchou ? Oui. Chouchou pousse la voiture sans presser. Les roues font un petit bruit. Le phare jaune avance. Elle va au rabat. Tu as entendu les roues ? Oui, papa. La voiture s'arrête devant le rabat. Le phare jaune touche le carton. Elle n'est pas dedans. Presque. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1643,7 +1664,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1651,10 +1672,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1677,30 +1698,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>proposer</t>
+          <t>Tu veux pousser</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1709,10 +1730,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1725,33 +1746,49 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_propose_mila_regarde; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou a su proposer.
-narrateur|Il accepte plusieurs réponses.
-enfant-m|D'accord.
-narrateur|Mila s'assoit près du mur.
-narrateur|Elle regarde la voiture.
-narrateur|Chouchou pousse la voiture.
+          <t>narrateur|Chouchou avance la voiture trop vite.
+enfant-f|Tu pousses, Mila, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+copine|Non.
+narrateur|Mila reste près du mur.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Chouchou refuse de foncer.
+narrateur|Elle lâche la manche, un peu.
+papa|La voiture est dehors, Chouchou ?
+narrateur|Papa reste à sa hauteur.
+maman|Le rabat est dur, sous tes mains.
+narrateur|Maman n'a pas fini non plus.
+narrateur|Chouchou attend que le silence arrive.
+enfant-f|Tu veux pousser ?
+narrateur|Mila ne dit rien.
+narrateur|Elle s'assoit près du mur.
+copine|Je regarde.
+enfant-f|D'accord.
+papa|Merci, Chouchou.
+narrateur|Papa a entendu toute la phrase.
+maman|Tu tiens la voiture des deux mains ?
+enfant-f|Oui, maman.
+enfant-f|Les roues sont froides.
+papa|Tu parles du vent, si tu veux ?
+enfant-f|La cheminée boit le vent.
+maman|On reste au couloir, Chouchou ?
+enfant-f|Oui.
+narrateur|Chouchou pousse la voiture sans presser.
 narrateur|Les roues font un petit bruit.
 narrateur|Le phare jaune avance.
+enfant-f|Elle va au rabat.
 papa|Tu as entendu les roues ?
-enfant-m|Oui, papa.
-enfant-m|Tu veux pousser ?
-copine|Plus tard.
-enfant-m|D'accord.
-maman|Plusieurs réponses sont possibles.
+enfant-f|Oui, papa.
 narrateur|La voiture s'arrête devant le rabat.
 narrateur|Le phare jaune touche le carton.
-narrateur|Elle n'est pas encore dedans.
-papa|Tu as plié le rabat.
-enfant-m|Deux fois.
-narrateur|Mila avance un peu.
-narrateur|Elle reste à regarder.
-maman|C'est bien.</t>
+narrateur|Elle n'est pas dedans.
+enfant-f|Presque.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1783,17 +1820,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou pousse encore. La voiture rentre. Les roues passent le rabat. Ça fait toc. Elle est dedans. Tu as accepté, Chouchou ? Oui, papa. Bravo. Il ferme le rabat. Le carton redevient calme. On n'entend plus les roues. J'ai regardé. Oui. Regarder, c'est une réponse. On range la voiture ? Elle dort déjà. Tu as fini le garage ? Oui, papa. Le vent chante encore, tout loin. Les rayures de Mila brillent. Le trait bleu du carton reste. La poussière est retombée.</t>
+          <t>Chouchou quitte le mur avec la voiture. Le vent glisse dans la cheminée. Tu fermes le rabat, maintenant ! Chouchou pousse trop vite. La voiture dépasse le carton. Oh. Papa n'a pas fini sa phrase. La voiture file, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le couloir, un instant. Elle observe la voiture, écoute la cheminée. Sur la brique, un éclat de cheminée luit. Il est là. Tu fermes le rabat, si tu veux ? Plus tard. D'accord. Mila reste à regarder. Chouchou pose la voiture sans presser. Les roues passent le rabat. Ça fait toc. Elle est dedans. Tu restes un peu ? Oui, papa. Le carton est près du mur. On le laisse ? Oui, contre la brique. La voiture sent le bois. Elle colle aux doigts. Comme le papier, oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Chouchou pousse encore. La voiture rentre. Les roues passent le rabat. Ça fait toc. Elle est dedans. Tu as accepté, Chouchou ? Oui, papa. Bravo. Il ferme le rabat. Le carton redevient calme. On n'entend plus les roues. J'ai regardé. Oui. Regarder, c'est une réponse. On range la voiture ? Elle dort déjà. Tu as fini le garage ? Oui, papa. Le vent chante encore, tout loin. Les rayures de Mila brillent. Le trait bleu du carton reste. La poussière est retombée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Chouchou quitte le mur avec la voiture. Le vent glisse dans la cheminée. Tu fermes le rabat, maintenant ! Chouchou pousse trop vite. La voiture dépasse le carton. Oh. Papa n'a pas fini sa phrase. La voiture file, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le couloir, un instant. Elle observe la voiture, écoute la cheminée. Sur la brique, un &lt;emphasis level="moderate"&gt;éclat de cheminée&lt;/emphasis&gt; luit. Il est là. Tu fermes le rabat, si tu veux ? Plus tard. D'accord. Mila reste à regarder. Chouchou pose la voiture sans presser. Les roues passent le rabat. Ça fait toc. Elle est dedans. Tu restes un peu ? Oui, papa. Le carton est près du mur. On le laisse ? Oui, contre la brique. La voiture sent le bois. Elle colle aux doigts. Comme le papier, oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Maman dit : on range. Kilian met un coussin. Maël met un coussin. Ils se disent merci. [pause]</t>
+          <t>Chouchou quitte le mur avec la voiture. Le vent glisse dans la cheminée. Tu fermes le rabat, maintenant ! Chouchou pousse trop vite. La voiture dépasse le carton. Oh. Papa n'a pas fini sa phrase. La voiture file, Chouchou. Les deux voix se mélangent. Oh. Chouchou refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Elle écoute le couloir, un instant. Elle observe la voiture, écoute la cheminée. Sur la brique, un &lt;emphasis&gt;éclat de cheminée&lt;/emphasis&gt; luit. Il est là. Tu fermes le rabat, si tu veux ? Plus tard. D'accord. Mila reste à regarder. Chouchou pose la voiture sans presser. Les roues passent le rabat. Ça fait toc. Elle est dedans. Tu restes un peu ? Oui, papa. Le carton est près du mur. On le laisse ? Oui, contre la brique. La voiture sent le bois. Elle colle aux doigts. Comme le papier, oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1840,7 +1877,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1848,10 +1885,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1872,28 +1909,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cheminée</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1902,10 +1943,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1916,31 +1957,45 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_sur_le_rabat; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Chouchou pousse encore.
-narrateur|La voiture rentre.
+          <t>narrateur|Chouchou quitte le mur avec la voiture.
+narrateur|Le vent glisse dans la cheminée.
+enfant-f|Tu fermes le rabat, maintenant !
+narrateur|Chouchou pousse trop vite.
+narrateur|La voiture dépasse le carton.
+enfant-f|Oh.
+narrateur|Papa n'a pas fini sa phrase.
+papa|La voiture file, Chouchou.
+narrateur|Les deux voix se mélangent.
+enfant-f|Oh.
+narrateur|Chouchou refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Elle écoute le couloir, un instant.
+narrateur|Elle observe la voiture, écoute la cheminée.
+narrateur|Sur la brique, un éclat de cheminée luit.
+enfant-f|Il est là.
+enfant-f|Tu fermes le rabat, si tu veux ?
+copine|Plus tard.
+enfant-f|D'accord.
+narrateur|Mila reste à regarder.
+narrateur|Chouchou pose la voiture sans presser.
 narrateur|Les roues passent le rabat.
 narrateur|Ça fait toc.
-enfant-m|Elle est dedans.
-papa|Tu as accepté, Chouchou ?
-enfant-m|Oui, papa.
-maman|Bravo.
-narrateur|Il ferme le rabat.
-narrateur|Le carton redevient calme.
-narrateur|On n'entend plus les roues.
-copine|J'ai regardé.
-papa|Oui.
-papa|Regarder, c'est une réponse.
-maman|On range la voiture ?
-enfant-m|Elle dort déjà.
-papa|Tu as fini le garage ?
-enfant-m|Oui, papa.
-narrateur|Le vent chante encore, tout loin.
-narrateur|Les rayures de Mila brillent.
-narrateur|Le trait bleu du carton reste.
-narrateur|La poussière est retombée.</t>
+enfant-f|Elle est dedans.
+papa|Tu restes un peu ?
+enfant-f|Oui, papa.
+maman|Le carton est près du mur.
+enfant-f|On le laisse ?
+papa|Oui, contre la brique.
+narrateur|La voiture sent le bois.
+enfant-f|Elle colle aux doigts.
+maman|Comme le papier, oui.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1972,17 +2027,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La voiture rouge dort dans le carton. Le phare jaune ne se voit plus. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. Le vent finit sa chanson.</t>
+          <t>Ils restent près du carton. Maman referme le rabat, sans bruit. Comme une porte, papa. Tu le vois, toi ? Oui, sur la brique. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le rabat est fermé, Chouchou. Oui, avec la voiture. L'odeur de papier reste dans le couloir. Il est là, maman. Oui, sur la brique. L'éclat de cheminée tient sur la brique.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La voiture rouge dort dans le carton. Le phare jaune ne se voit plus. J'ai proposé. J'ai accepté. Plusieurs réponses sont possibles. Oui. Le vent finit sa chanson.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du carton. Maman referme le rabat, sans bruit. Comme une porte, papa. Tu le vois, toi ? Oui, sur la brique. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le rabat est fermé, Chouchou. Oui, avec la voiture. L'odeur de papier reste dans le couloir. Il est là, maman. Oui, sur la brique. L'&lt;emphasis level="moderate"&gt;éclat de cheminée&lt;/emphasis&gt; tient sur la brique.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du carton. Maman referme le rabat, sans bruit. Comme une porte, papa. Tu le vois, toi ? Oui, sur la brique. On est bien, ici. Chouchou glisse le doigt, sans se presser. On le sent, maman. Tu le sens sur tes doigts ? Oui, il colle. Le rabat est fermé, Chouchou. Oui, avec la voiture. L'odeur de papier reste dans le couloir. Il est là, maman. Oui, sur la brique. L'&lt;emphasis&gt;éclat de cheminée&lt;/emphasis&gt; tient sur la brique.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2029,18 +2084,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2049,12 +2104,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2063,17 +2118,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de cheminée</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2082,11 +2141,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2095,30 +2154,48 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse et fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_la_brique; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La voiture rouge dort dans le carton.
-narrateur|Le phare jaune ne se voit plus.
-enfant-m|J'ai proposé.
-enfant-m|J'ai accepté.
-maman|Plusieurs réponses sont possibles.
-papa|Oui.
-narrateur|Le vent finit sa chanson.</t>
+          <t>narrateur|Ils restent près du carton.
+narrateur|Maman referme le rabat, sans bruit.
+enfant-f|Comme une porte, papa.
+papa|Tu le vois, toi ?
+enfant-f|Oui, sur la brique.
+maman|On est bien, ici.
+narrateur|Chouchou glisse le doigt, sans se presser.
+enfant-f|On le sent, maman.
+maman|Tu le sens sur tes doigts ?
+enfant-f|Oui, il colle.
+papa|Le rabat est fermé, Chouchou.
+enfant-f|Oui, avec la voiture.
+narrateur|L'odeur de papier reste dans le couloir.
+enfant-f|Il est là, maman.
+maman|Oui, sur la brique.
+narrateur|L'éclat de cheminée tient sur la brique.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>vent</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2216,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A11"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2217,6 +2294,13 @@
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>